<commit_message>
Updated names, model & article discrepancies
</commit_message>
<xml_diff>
--- a/public/COIN Model.xlsx
+++ b/public/COIN Model.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sidshah/Library/Mobile Documents/com~apple~CloudDocs/Projects/Coinbase Research/Phase 3 - Consolidation &amp; Modeling/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2C0A463-0AE0-BA46-8BC4-267BF77D9622}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16AC8548-ECB5-A745-BCD7-42BA43EBE724}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="21000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3948,6 +3948,8 @@
     <xf numFmtId="0" fontId="101" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="73" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="74" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="38" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -3992,8 +3994,6 @@
     </xf>
     <xf numFmtId="0" fontId="64" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="13" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="73" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="74" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="fa_column_header_top_left" xfId="1" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
@@ -4824,12 +4824,12 @@
       <c r="B42" s="53" t="s">
         <v>320</v>
       </c>
-      <c r="C42" s="523" t="s">
+      <c r="C42" s="525" t="s">
         <v>321</v>
       </c>
-      <c r="D42" s="524"/>
-      <c r="E42" s="524"/>
-      <c r="F42" s="523"/>
+      <c r="D42" s="526"/>
+      <c r="E42" s="526"/>
+      <c r="F42" s="525"/>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43" s="52"/>
@@ -4846,12 +4846,12 @@
       <c r="B44" s="43" t="s">
         <v>336</v>
       </c>
-      <c r="C44" s="517" t="s">
+      <c r="C44" s="519" t="s">
         <v>558</v>
       </c>
-      <c r="D44" s="517"/>
-      <c r="E44" s="517"/>
-      <c r="F44" s="518"/>
+      <c r="D44" s="519"/>
+      <c r="E44" s="519"/>
+      <c r="F44" s="520"/>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A45" s="52"/>
@@ -4868,36 +4868,36 @@
       <c r="B46" s="42" t="s">
         <v>337</v>
       </c>
-      <c r="C46" s="525" t="s">
+      <c r="C46" s="527" t="s">
         <v>324</v>
       </c>
-      <c r="D46" s="525"/>
-      <c r="E46" s="525"/>
-      <c r="F46" s="526"/>
+      <c r="D46" s="527"/>
+      <c r="E46" s="527"/>
+      <c r="F46" s="528"/>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A47" s="52"/>
       <c r="B47" s="79" t="s">
         <v>338</v>
       </c>
-      <c r="C47" s="527" t="s">
+      <c r="C47" s="529" t="s">
         <v>325</v>
       </c>
-      <c r="D47" s="527"/>
-      <c r="E47" s="527"/>
-      <c r="F47" s="528"/>
+      <c r="D47" s="529"/>
+      <c r="E47" s="529"/>
+      <c r="F47" s="530"/>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A48" s="52"/>
       <c r="B48" s="80" t="s">
         <v>339</v>
       </c>
-      <c r="C48" s="519" t="s">
+      <c r="C48" s="521" t="s">
         <v>326</v>
       </c>
-      <c r="D48" s="519"/>
-      <c r="E48" s="519"/>
-      <c r="F48" s="520"/>
+      <c r="D48" s="521"/>
+      <c r="E48" s="521"/>
+      <c r="F48" s="522"/>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A49" s="52"/>
@@ -4914,12 +4914,12 @@
       <c r="B50" s="78" t="s">
         <v>340</v>
       </c>
-      <c r="C50" s="515" t="s">
+      <c r="C50" s="517" t="s">
         <v>369</v>
       </c>
-      <c r="D50" s="515"/>
-      <c r="E50" s="515"/>
-      <c r="F50" s="516"/>
+      <c r="D50" s="517"/>
+      <c r="E50" s="517"/>
+      <c r="F50" s="518"/>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A51" s="52"/>
@@ -4936,24 +4936,24 @@
       <c r="B52" s="43" t="s">
         <v>341</v>
       </c>
-      <c r="C52" s="517" t="s">
+      <c r="C52" s="519" t="s">
         <v>370</v>
       </c>
-      <c r="D52" s="517"/>
-      <c r="E52" s="517"/>
-      <c r="F52" s="518"/>
+      <c r="D52" s="519"/>
+      <c r="E52" s="519"/>
+      <c r="F52" s="520"/>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A53" s="52"/>
       <c r="B53" s="80" t="s">
         <v>342</v>
       </c>
-      <c r="C53" s="519" t="s">
+      <c r="C53" s="521" t="s">
         <v>329</v>
       </c>
-      <c r="D53" s="519"/>
-      <c r="E53" s="519"/>
-      <c r="F53" s="520"/>
+      <c r="D53" s="521"/>
+      <c r="E53" s="521"/>
+      <c r="F53" s="522"/>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A54" s="52"/>
@@ -4970,12 +4970,12 @@
       <c r="B55" s="61" t="s">
         <v>343</v>
       </c>
-      <c r="C55" s="521" t="s">
+      <c r="C55" s="523" t="s">
         <v>331</v>
       </c>
-      <c r="D55" s="521"/>
-      <c r="E55" s="521"/>
-      <c r="F55" s="522"/>
+      <c r="D55" s="523"/>
+      <c r="E55" s="523"/>
+      <c r="F55" s="524"/>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A56" s="52"/>
@@ -5060,42 +5060,42 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="21" x14ac:dyDescent="0.25">
-      <c r="A1" s="529" t="s">
+      <c r="A1" s="531" t="s">
         <v>195</v>
       </c>
-      <c r="B1" s="529"/>
-      <c r="C1" s="529"/>
-      <c r="D1" s="529"/>
-      <c r="E1" s="529"/>
-      <c r="F1" s="529"/>
-      <c r="G1" s="529"/>
-      <c r="H1" s="529"/>
-      <c r="I1" s="529"/>
-      <c r="J1" s="529"/>
-      <c r="K1" s="529"/>
-      <c r="L1" s="529"/>
-      <c r="M1" s="529"/>
-      <c r="N1" s="529"/>
-      <c r="O1" s="529"/>
-      <c r="P1" s="529"/>
+      <c r="B1" s="531"/>
+      <c r="C1" s="531"/>
+      <c r="D1" s="531"/>
+      <c r="E1" s="531"/>
+      <c r="F1" s="531"/>
+      <c r="G1" s="531"/>
+      <c r="H1" s="531"/>
+      <c r="I1" s="531"/>
+      <c r="J1" s="531"/>
+      <c r="K1" s="531"/>
+      <c r="L1" s="531"/>
+      <c r="M1" s="531"/>
+      <c r="N1" s="531"/>
+      <c r="O1" s="531"/>
+      <c r="P1" s="531"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A2" s="530"/>
-      <c r="B2" s="530"/>
-      <c r="C2" s="530"/>
-      <c r="D2" s="530"/>
-      <c r="E2" s="530"/>
-      <c r="F2" s="530"/>
-      <c r="G2" s="530"/>
-      <c r="H2" s="530"/>
-      <c r="I2" s="530"/>
-      <c r="J2" s="530"/>
-      <c r="K2" s="530"/>
-      <c r="L2" s="530"/>
-      <c r="M2" s="530"/>
-      <c r="N2" s="530"/>
-      <c r="O2" s="530"/>
-      <c r="P2" s="530"/>
+      <c r="A2" s="532"/>
+      <c r="B2" s="532"/>
+      <c r="C2" s="532"/>
+      <c r="D2" s="532"/>
+      <c r="E2" s="532"/>
+      <c r="F2" s="532"/>
+      <c r="G2" s="532"/>
+      <c r="H2" s="532"/>
+      <c r="I2" s="532"/>
+      <c r="J2" s="532"/>
+      <c r="K2" s="532"/>
+      <c r="L2" s="532"/>
+      <c r="M2" s="532"/>
+      <c r="N2" s="532"/>
+      <c r="O2" s="532"/>
+      <c r="P2" s="532"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3" s="178"/>
@@ -5395,7 +5395,7 @@
         <v>93500</v>
       </c>
       <c r="D11" s="257">
-        <v>96500</v>
+        <v>87000</v>
       </c>
       <c r="E11" s="445">
         <v>80000</v>
@@ -18888,38 +18888,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="20" x14ac:dyDescent="0.2">
-      <c r="A1" s="531" t="s">
+      <c r="A1" s="515" t="s">
         <v>539</v>
       </c>
-      <c r="B1" s="531"/>
-      <c r="C1" s="531"/>
-      <c r="D1" s="531"/>
-      <c r="E1" s="531"/>
-      <c r="F1" s="531"/>
-      <c r="G1" s="531"/>
-      <c r="H1" s="531"/>
-      <c r="I1" s="531"/>
-      <c r="J1" s="531"/>
-      <c r="K1" s="531"/>
-      <c r="L1" s="531"/>
-      <c r="M1" s="531"/>
-      <c r="N1" s="531"/>
+      <c r="B1" s="515"/>
+      <c r="C1" s="515"/>
+      <c r="D1" s="515"/>
+      <c r="E1" s="515"/>
+      <c r="F1" s="515"/>
+      <c r="G1" s="515"/>
+      <c r="H1" s="515"/>
+      <c r="I1" s="515"/>
+      <c r="J1" s="515"/>
+      <c r="K1" s="515"/>
+      <c r="L1" s="515"/>
+      <c r="M1" s="515"/>
+      <c r="N1" s="515"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A2" s="532"/>
-      <c r="B2" s="532"/>
-      <c r="C2" s="532"/>
-      <c r="D2" s="532"/>
-      <c r="E2" s="532"/>
-      <c r="F2" s="532"/>
-      <c r="G2" s="532"/>
-      <c r="H2" s="532"/>
-      <c r="I2" s="532"/>
-      <c r="J2" s="532"/>
-      <c r="K2" s="532"/>
-      <c r="L2" s="532"/>
-      <c r="M2" s="532"/>
-      <c r="N2" s="532"/>
+      <c r="A2" s="516"/>
+      <c r="B2" s="516"/>
+      <c r="C2" s="516"/>
+      <c r="D2" s="516"/>
+      <c r="E2" s="516"/>
+      <c r="F2" s="516"/>
+      <c r="G2" s="516"/>
+      <c r="H2" s="516"/>
+      <c r="I2" s="516"/>
+      <c r="J2" s="516"/>
+      <c r="K2" s="516"/>
+      <c r="L2" s="516"/>
+      <c r="M2" s="516"/>
+      <c r="N2" s="516"/>
     </row>
     <row r="3" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="359" t="s">

</xml_diff>